<commit_message>
DP - create ministry_of_education_coordinates file
</commit_message>
<xml_diff>
--- a/utils/Intermediates/250121_BShemesh_moe_mosdot_coordinates_2022.xlsx
+++ b/utils/Intermediates/250121_BShemesh_moe_mosdot_coordinates_2022.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F161"/>
+  <dimension ref="A1:G161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,6 +459,11 @@
           <t>coordinate_y</t>
         </is>
       </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SRC</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -485,6 +490,11 @@
       <c r="F2" t="n">
         <v>628087</v>
       </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -511,6 +521,11 @@
       <c r="F3" t="n">
         <v>627529</v>
       </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -537,6 +552,11 @@
       <c r="F4" t="n">
         <v>628865</v>
       </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -563,6 +583,11 @@
       <c r="F5" t="n">
         <v>627534</v>
       </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -589,6 +614,11 @@
       <c r="F6" t="n">
         <v>627493</v>
       </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -615,6 +645,11 @@
       <c r="F7" t="n">
         <v>628208</v>
       </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -641,6 +676,11 @@
       <c r="F8" t="n">
         <v>627176</v>
       </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -667,6 +707,11 @@
       <c r="F9" t="n">
         <v>627517</v>
       </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -693,6 +738,11 @@
       <c r="F10" t="n">
         <v>627650</v>
       </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -719,6 +769,11 @@
       <c r="F11" t="n">
         <v>627750</v>
       </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -745,6 +800,11 @@
       <c r="F12" t="n">
         <v>627640</v>
       </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -771,6 +831,11 @@
       <c r="F13" t="n">
         <v>625914</v>
       </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -797,6 +862,11 @@
       <c r="F14" t="n">
         <v>627248</v>
       </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -823,6 +893,11 @@
       <c r="F15" t="n">
         <v>627524</v>
       </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -849,6 +924,11 @@
       <c r="F16" t="n">
         <v>626478</v>
       </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -875,6 +955,11 @@
       <c r="F17" t="n">
         <v>628214</v>
       </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -901,6 +986,11 @@
       <c r="F18" t="n">
         <v>628818</v>
       </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -927,6 +1017,11 @@
       <c r="F19" t="n">
         <v>624471</v>
       </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -953,6 +1048,11 @@
       <c r="F20" t="n">
         <v>625920</v>
       </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -979,6 +1079,11 @@
       <c r="F21" t="n">
         <v>627712</v>
       </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -1005,6 +1110,11 @@
       <c r="F22" t="n">
         <v>624915</v>
       </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -1031,6 +1141,11 @@
       <c r="F23" t="n">
         <v>628256</v>
       </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -1057,6 +1172,11 @@
       <c r="F24" t="n">
         <v>625878</v>
       </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -1083,6 +1203,11 @@
       <c r="F25" t="n">
         <v>628018</v>
       </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1109,6 +1234,11 @@
       <c r="F26" t="n">
         <v>624811</v>
       </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1135,6 +1265,11 @@
       <c r="F27" t="n">
         <v>624175</v>
       </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1161,6 +1296,11 @@
       <c r="F28" t="n">
         <v>625914</v>
       </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1187,6 +1327,11 @@
       <c r="F29" t="n">
         <v>624080</v>
       </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1213,6 +1358,11 @@
       <c r="F30" t="n">
         <v>624086</v>
       </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1239,6 +1389,11 @@
       <c r="F31" t="n">
         <v>624876</v>
       </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1265,6 +1420,11 @@
       <c r="F32" t="n">
         <v>627386</v>
       </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1291,6 +1451,11 @@
       <c r="F33" t="n">
         <v>624081</v>
       </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1317,6 +1482,11 @@
       <c r="F34" t="n">
         <v>625967</v>
       </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1343,6 +1513,11 @@
       <c r="F35" t="n">
         <v>627208</v>
       </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1369,6 +1544,11 @@
       <c r="F36" t="n">
         <v>627750</v>
       </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1395,6 +1575,11 @@
       <c r="F37" t="n">
         <v>627946</v>
       </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1421,6 +1606,11 @@
       <c r="F38" t="n">
         <v>624128</v>
       </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1447,6 +1637,11 @@
       <c r="F39" t="n">
         <v>624783</v>
       </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1473,6 +1668,11 @@
       <c r="F40" t="n">
         <v>627103</v>
       </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1499,6 +1699,11 @@
       <c r="F41" t="n">
         <v>624877</v>
       </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1525,6 +1730,11 @@
       <c r="F42" t="n">
         <v>624876</v>
       </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1551,6 +1761,11 @@
       <c r="F43" t="n">
         <v>628374</v>
       </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
@@ -1577,6 +1792,11 @@
       <c r="F44" t="n">
         <v>624514</v>
       </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
@@ -1603,6 +1823,11 @@
       <c r="F45" t="n">
         <v>624186</v>
       </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
@@ -1629,6 +1854,11 @@
       <c r="F46" t="n">
         <v>625914</v>
       </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1655,6 +1885,11 @@
       <c r="F47" t="n">
         <v>624168</v>
       </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1681,6 +1916,11 @@
       <c r="F48" t="n">
         <v>628208</v>
       </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1707,6 +1947,11 @@
       <c r="F49" t="n">
         <v>624047</v>
       </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1733,6 +1978,11 @@
       <c r="F50" t="n">
         <v>624783</v>
       </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1759,6 +2009,11 @@
       <c r="F51" t="n">
         <v>624492</v>
       </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1785,6 +2040,11 @@
       <c r="F52" t="n">
         <v>624851</v>
       </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1811,6 +2071,11 @@
       <c r="F53" t="n">
         <v>625922</v>
       </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1837,6 +2102,11 @@
       <c r="F54" t="n">
         <v>626913</v>
       </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1863,6 +2133,11 @@
       <c r="F55" t="n">
         <v>627454</v>
       </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1889,6 +2164,11 @@
       <c r="F56" t="n">
         <v>624222</v>
       </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1915,6 +2195,11 @@
       <c r="F57" t="n">
         <v>623372</v>
       </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1941,6 +2226,11 @@
       <c r="F58" t="n">
         <v>628290</v>
       </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1967,6 +2257,11 @@
       <c r="F59" t="n">
         <v>625692</v>
       </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1993,6 +2288,11 @@
       <c r="F60" t="n">
         <v>624630</v>
       </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -2019,6 +2319,11 @@
       <c r="F61" t="n">
         <v>624876</v>
       </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -2045,6 +2350,11 @@
       <c r="F62" t="n">
         <v>624630</v>
       </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -2071,6 +2381,11 @@
       <c r="F63" t="n">
         <v>626477</v>
       </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -2097,6 +2412,11 @@
       <c r="F64" t="n">
         <v>626694</v>
       </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -2123,6 +2443,11 @@
       <c r="F65" t="n">
         <v>624804</v>
       </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -2149,6 +2474,11 @@
       <c r="F66" t="n">
         <v>624137</v>
       </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -2175,6 +2505,11 @@
       <c r="F67" t="n">
         <v>627423</v>
       </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -2201,6 +2536,11 @@
       <c r="F68" t="n">
         <v>624572</v>
       </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="n">
@@ -2227,6 +2567,11 @@
       <c r="F69" t="n">
         <v>627238</v>
       </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -2253,6 +2598,11 @@
       <c r="F70" t="n">
         <v>627243</v>
       </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2279,6 +2629,11 @@
       <c r="F71" t="n">
         <v>623686</v>
       </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2305,6 +2660,11 @@
       <c r="F72" t="n">
         <v>624289</v>
       </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2331,6 +2691,11 @@
       <c r="F73" t="n">
         <v>628635</v>
       </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2357,6 +2722,11 @@
       <c r="F74" t="n">
         <v>624082</v>
       </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2383,6 +2753,11 @@
       <c r="F75" t="n">
         <v>624632</v>
       </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2409,6 +2784,11 @@
       <c r="F76" t="n">
         <v>627203</v>
       </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2435,6 +2815,11 @@
       <c r="F77" t="n">
         <v>623893</v>
       </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2461,6 +2846,11 @@
       <c r="F78" t="n">
         <v>628283</v>
       </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="n">
@@ -2487,6 +2877,11 @@
       <c r="F79" t="n">
         <v>624305</v>
       </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="n">
@@ -2513,6 +2908,11 @@
       <c r="F80" t="n">
         <v>624804</v>
       </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="n">
@@ -2539,6 +2939,11 @@
       <c r="F81" t="n">
         <v>625615</v>
       </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="n">
@@ -2565,6 +2970,11 @@
       <c r="F82" t="n">
         <v>626694</v>
       </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="n">
@@ -2591,6 +3001,11 @@
       <c r="F83" t="n">
         <v>628238</v>
       </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="n">
@@ -2617,6 +3032,11 @@
       <c r="F84" t="n">
         <v>628735</v>
       </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="n">
@@ -2643,6 +3063,11 @@
       <c r="F85" t="n">
         <v>626630</v>
       </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="n">
@@ -2669,6 +3094,11 @@
       <c r="F86" t="n">
         <v>624293</v>
       </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="n">
@@ -2695,6 +3125,11 @@
       <c r="F87" t="n">
         <v>627379</v>
       </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="n">
@@ -2721,6 +3156,11 @@
       <c r="F88" t="n">
         <v>627866</v>
       </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="n">
@@ -2747,6 +3187,11 @@
       <c r="F89" t="n">
         <v>624933</v>
       </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="n">
@@ -2773,6 +3218,11 @@
       <c r="F90" t="n">
         <v>624572</v>
       </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="n">
@@ -2799,6 +3249,11 @@
       <c r="F91" t="n">
         <v>624876</v>
       </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="n">
@@ -2825,6 +3280,11 @@
       <c r="F92" t="n">
         <v>627441</v>
       </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="n">
@@ -2851,6 +3311,11 @@
       <c r="F93" t="n">
         <v>624220</v>
       </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="n">
@@ -2877,6 +3342,11 @@
       <c r="F94" t="n">
         <v>627648</v>
       </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="n">
@@ -2903,6 +3373,11 @@
       <c r="F95" t="n">
         <v>624771</v>
       </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="n">
@@ -2929,6 +3404,11 @@
       <c r="F96" t="n">
         <v>624250</v>
       </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="n">
@@ -2955,6 +3435,11 @@
       <c r="F97" t="n">
         <v>627874</v>
       </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="n">
@@ -2981,6 +3466,11 @@
       <c r="F98" t="n">
         <v>627937</v>
       </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="n">
@@ -3007,6 +3497,11 @@
       <c r="F99" t="n">
         <v>628671</v>
       </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="n">
@@ -3033,6 +3528,11 @@
       <c r="F100" t="n">
         <v>627379</v>
       </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="n">
@@ -3059,6 +3559,11 @@
       <c r="F101" t="n">
         <v>627927</v>
       </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="n">
@@ -3085,6 +3590,11 @@
       <c r="F102" t="n">
         <v>626463</v>
       </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="n">
@@ -3111,6 +3621,11 @@
       <c r="F103" t="n">
         <v>623880</v>
       </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="n">
@@ -3137,6 +3652,11 @@
       <c r="F104" t="n">
         <v>625939</v>
       </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="n">
@@ -3163,6 +3683,11 @@
       <c r="F105" t="n">
         <v>628701</v>
       </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="n">
@@ -3189,6 +3714,11 @@
       <c r="F106" t="n">
         <v>628733</v>
       </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="n">
@@ -3215,6 +3745,11 @@
       <c r="F107" t="n">
         <v>624771</v>
       </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="n">
@@ -3241,6 +3776,11 @@
       <c r="F108" t="n">
         <v>624262</v>
       </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="n">
@@ -3267,6 +3807,11 @@
       <c r="F109" t="n">
         <v>624487</v>
       </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="n">
@@ -3293,6 +3838,11 @@
       <c r="F110" t="n">
         <v>623605</v>
       </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="n">
@@ -3319,6 +3869,11 @@
       <c r="F111" t="n">
         <v>627063</v>
       </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="n">
@@ -3345,6 +3900,11 @@
       <c r="F112" t="n">
         <v>627795</v>
       </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="n">
@@ -3371,6 +3931,11 @@
       <c r="F113" t="n">
         <v>627238</v>
       </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="n">
@@ -3397,6 +3962,11 @@
       <c r="F114" t="n">
         <v>623851</v>
       </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="n">
@@ -3423,6 +3993,11 @@
       <c r="F115" t="n">
         <v>628791</v>
       </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="n">
@@ -3449,6 +4024,11 @@
       <c r="F116" t="n">
         <v>627063</v>
       </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="n">
@@ -3475,6 +4055,11 @@
       <c r="F117" t="n">
         <v>625286</v>
       </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="n">
@@ -3501,6 +4086,11 @@
       <c r="F118" t="n">
         <v>627968</v>
       </c>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="n">
@@ -3527,6 +4117,11 @@
       <c r="F119" t="n">
         <v>623623</v>
       </c>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="n">
@@ -3553,6 +4148,11 @@
       <c r="F120" t="n">
         <v>623623</v>
       </c>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="n">
@@ -3579,6 +4179,11 @@
       <c r="F121" t="n">
         <v>627238</v>
       </c>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="n">
@@ -3605,6 +4210,11 @@
       <c r="F122" t="n">
         <v>623426</v>
       </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="n">
@@ -3631,6 +4241,11 @@
       <c r="F123" t="n">
         <v>623921</v>
       </c>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="n">
@@ -3657,6 +4272,11 @@
       <c r="F124" t="n">
         <v>623921</v>
       </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="n">
@@ -3683,6 +4303,11 @@
       <c r="F125" t="n">
         <v>624376</v>
       </c>
+      <c r="G125" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="n">
@@ -3709,6 +4334,11 @@
       <c r="F126" t="n">
         <v>624848</v>
       </c>
+      <c r="G126" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="n">
@@ -3735,6 +4365,11 @@
       <c r="F127" t="n">
         <v>628209</v>
       </c>
+      <c r="G127" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="n">
@@ -3761,6 +4396,11 @@
       <c r="F128" t="n">
         <v>628585</v>
       </c>
+      <c r="G128" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="n">
@@ -3787,6 +4427,11 @@
       <c r="F129" t="n">
         <v>628657</v>
       </c>
+      <c r="G129" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="n">
@@ -3813,6 +4458,11 @@
       <c r="F130" t="n">
         <v>626655</v>
       </c>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="n">
@@ -3839,6 +4489,11 @@
       <c r="F131" t="n">
         <v>627238</v>
       </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="n">
@@ -3865,6 +4520,11 @@
       <c r="F132" t="n">
         <v>627063</v>
       </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="n">
@@ -3891,6 +4551,11 @@
       <c r="F133" t="n">
         <v>626750</v>
       </c>
+      <c r="G133" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="n">
@@ -3917,6 +4582,11 @@
       <c r="F134" t="n">
         <v>623850</v>
       </c>
+      <c r="G134" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="n">
@@ -3943,6 +4613,11 @@
       <c r="F135" t="n">
         <v>624634</v>
       </c>
+      <c r="G135" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="n">
@@ -3969,6 +4644,11 @@
       <c r="F136" t="n">
         <v>624277</v>
       </c>
+      <c r="G136" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="n">
@@ -3995,6 +4675,11 @@
       <c r="F137" t="n">
         <v>623615</v>
       </c>
+      <c r="G137" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="n">
@@ -4021,6 +4706,11 @@
       <c r="F138" t="n">
         <v>623426</v>
       </c>
+      <c r="G138" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="n">
@@ -4047,6 +4737,11 @@
       <c r="F139" t="n">
         <v>627480</v>
       </c>
+      <c r="G139" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="n">
@@ -4073,6 +4768,11 @@
       <c r="F140" t="n">
         <v>627238</v>
       </c>
+      <c r="G140" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="n">
@@ -4099,6 +4799,11 @@
       <c r="F141" t="n">
         <v>627414</v>
       </c>
+      <c r="G141" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="n">
@@ -4125,6 +4830,11 @@
       <c r="F142" t="n">
         <v>624692</v>
       </c>
+      <c r="G142" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="n">
@@ -4151,6 +4861,11 @@
       <c r="F143" t="n">
         <v>623234</v>
       </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="n">
@@ -4177,6 +4892,11 @@
       <c r="F144" t="n">
         <v>623234</v>
       </c>
+      <c r="G144" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="n">
@@ -4203,6 +4923,11 @@
       <c r="F145" t="n">
         <v>623347</v>
       </c>
+      <c r="G145" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="n">
@@ -4229,6 +4954,11 @@
       <c r="F146" t="n">
         <v>626217</v>
       </c>
+      <c r="G146" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="n">
@@ -4255,6 +4985,11 @@
       <c r="F147" t="n">
         <v>624223</v>
       </c>
+      <c r="G147" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="n">
@@ -4281,6 +5016,11 @@
       <c r="F148" t="n">
         <v>623672</v>
       </c>
+      <c r="G148" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="n">
@@ -4307,6 +5047,11 @@
       <c r="F149" t="n">
         <v>628733</v>
       </c>
+      <c r="G149" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="n">
@@ -4333,6 +5078,11 @@
       <c r="F150" t="n">
         <v>627063</v>
       </c>
+      <c r="G150" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="n">
@@ -4359,6 +5109,11 @@
       <c r="F151" t="n">
         <v>627063</v>
       </c>
+      <c r="G151" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="n">
@@ -4385,6 +5140,11 @@
       <c r="F152" t="n">
         <v>623725</v>
       </c>
+      <c r="G152" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="n">
@@ -4411,6 +5171,11 @@
       <c r="F153" t="n">
         <v>628670</v>
       </c>
+      <c r="G153" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="n">
@@ -4437,6 +5202,11 @@
       <c r="F154" t="n">
         <v>623535</v>
       </c>
+      <c r="G154" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="n">
@@ -4463,6 +5233,11 @@
       <c r="F155" t="n">
         <v>628234</v>
       </c>
+      <c r="G155" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="n">
@@ -4489,6 +5264,11 @@
       <c r="F156" t="n">
         <v>627063</v>
       </c>
+      <c r="G156" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="n">
@@ -4515,6 +5295,11 @@
       <c r="F157" t="n">
         <v>623605</v>
       </c>
+      <c r="G157" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="n">
@@ -4541,6 +5326,11 @@
       <c r="F158" t="n">
         <v>625092</v>
       </c>
+      <c r="G158" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="159">
       <c r="A159" t="n">
@@ -4567,6 +5357,11 @@
       <c r="F159" t="n">
         <v>628733</v>
       </c>
+      <c r="G159" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="n">
@@ -4593,6 +5388,11 @@
       <c r="F160" t="n">
         <v>628936</v>
       </c>
+      <c r="G160" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="n">
@@ -4618,6 +5418,11 @@
       </c>
       <c r="F161" t="n">
         <v>627570</v>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>moe_mosdot_coordinates</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>